<commit_message>
Update test cases Excel file with modifications
</commit_message>
<xml_diff>
--- a/test_automation/Assignment 1 - Test cases.xlsx
+++ b/test_automation/Assignment 1 - Test cases.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name=" Test cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name=" Test cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,35 +27,26 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DEEAF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -68,10 +58,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -79,18 +78,18 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -454,13 +453,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="3" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
@@ -472,37 +469,37 @@
           <t>TC ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Input length type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Expected output</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Actual output</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Singlish input types covered</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Evidence or rationale for the input type covered</t>
         </is>
@@ -529,8 +526,16 @@
           <t>අපි කොහෙද යනවා?</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>අපි කොහෙද යනවා?</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Question forms</t>
@@ -543,34 +548,42 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Neg_0002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>oya danne ada office eka wela thiyenne kawda kiyala? mama check karanna hithuwa.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>ඔයා දන්නේ අද office එක වෙලා තියෙන්නේ කාවද කියලා? මම check කරන්න හිතුවා.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ඔයා දන්නේ අද office එක වෙලා තියෙන්නේ කව්ද කියලා? මම check කරන්න හිතුවා.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Question forms; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Rationale: Indirect question form; Evidence: 'office', 'check' are English words inserted</t>
         </is>
@@ -597,8 +610,16 @@
           <t>ඒක මට දෙන්න එපා.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>ඒක මට දෙන්න එපා.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Command forms</t>
@@ -611,34 +632,42 @@
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Neg_0004</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>potha tika table eke tiyala yanna, mama awith balamu.</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>පොත ටික table එකේ තියලා යන්න, මම ආවිත් බලමු.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>පොත ටික table එකේ තියලා යන්න, මම ඇවිත් බලමු.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Command forms; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Rationale: Imperative command sentence; Evidence: 'table' is an English word inserted</t>
         </is>
@@ -665,8 +694,16 @@
           <t>කොහොමද මචං, ගොඩක් කාලං නෑ!</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>කොහොමද මචං, ගොඩක් කලාම නැ!</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Greetings; Inputs with Slang and Casual Phrasing</t>
@@ -679,34 +716,42 @@
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Neg_0006</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>subha udaesanak wewa nangi! ada birthday eka nisa special dinner ekak gamu.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>සුභ උදෑසනක් වේවා නංගී! අද birthday එක නිසා special dinner එකක් යමු.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>සුභ උදෑසනක් වේවා නංගි! අද birthday එක නිසා special dinner එකක් ගමු.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Greetings; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Rationale: Morning greeting; Evidence: 'birthday', 'dinner', 'special' are English words</t>
         </is>
@@ -733,8 +778,16 @@
           <t>පොඩ්ඩක් මිනිස්සු වෙලා කතා කරන්න.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>පොඩ්ඩක් මිනිස්සු වෙලා කතා කරන්න.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Requests</t>
@@ -747,34 +800,42 @@
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Neg_0008</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>oyage number eka mata text ekak dannapan, mama miss call ekak dunna naeda oyata?</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>ඔයාගේ number එක මට text එකක් දන්නපං, මම miss call එකක් දුන්නා නෑද ඔයාට?</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>ඔයාගේ number එක මට text එකක් දාන්නපන්, මම miss call එකක් දුන්නා නේද ඔයාට?</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Requests; Platform/App Names in Singlish; English Digital Terms in Singlish</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Rationale: Request for contact; Evidence: 'text', 'number', 'miss call' are digital terms</t>
         </is>
@@ -801,8 +862,16 @@
           <t>නෑ නෑ, මම දන්නේ නෑ ඒක.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>නැ නැ, මම දන්නේ නෑ ඒක.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Responses</t>
@@ -815,34 +884,42 @@
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Neg_0010</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>hari, mama ekata agree, ane apita thamai ena kiyala hithuwe naeda.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>හරි, මම ඒකට agree, අනේ අපිටා තමයි එනා කියලා හිතුවේ නෑද.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>හරි, මම ඒකට agree, අනේ අපිට තමයි එන කියලා හිතුවේ නෑද.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Responses; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Rationale: Affirmative response; Evidence: 'agree' is an English word inserted</t>
         </is>
@@ -869,8 +946,16 @@
           <t>ආඩෝ ආඩෝ, අහේ බලා!</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>අඩො අඩො, අහේ බලා!</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Repeated Words; Inputs with Slang and Casual Phrasing</t>
@@ -883,34 +968,42 @@
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Neg_0012</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>poddak poddak ganna, nathnam amaru weyi, tika tika karamu.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>පොඩ්ඩක් පොඩ්ඩක් ගන්න, නැත්නම් අමාරු වෙයි, ටික ටික කරමු.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>පොඩ්ඩක් පොඩ්ඩක් ගන්න, නැත්නම් අමාරු වෙයි, ටික ටික කරමු.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Repeated Words</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Rationale: Multiple repeated words used for emphasis throughout</t>
         </is>
@@ -937,8 +1030,16 @@
           <t>අනේ! ඔයා කොහෙද ගියේ?</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>අනේ! ඔයා කොහෙද ගියේ?</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Inputs with Punctuation Marks; Question forms</t>
@@ -951,34 +1052,42 @@
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Neg_0014</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>mama yanawa... oya enawada? nathnam... mama ekka yanna.</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>මම යනවා... ඔයා එනවාද? නැත්නම්... මම එක්ක යන්න.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>මම යනවා... ඔයා එනවද? නැත්නම්... මම එක්ක යන්න.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Inputs with Punctuation Marks; Question forms</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Rationale: Uses ellipsis (...) and question mark (?)</t>
         </is>
@@ -1005,8 +1114,16 @@
           <t>මං ඔයාට පෙන්නා පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>මන් ඔයාට පෙන්නන්න පුළුවන්ද?</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Romanization / Spelling Variants; Question forms</t>
@@ -1019,34 +1136,42 @@
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Neg_0016</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>machang mta adha pass wenm namk dagnn, karunakrla hlp krnn.</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>මචං මට අද pass වෙන්නම් නමක් දාගන්න, කරුණාකරලා help කරන්න.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>මචං මට අද පාස් වෙනම නමක් දාගන්න, කරුණාකරලා බලපන් කරන්න.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Romanization / Spelling Variants; Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Rationale: Heavily abbreviated spelling throughout; 'machang' variant spelling of 'machan'</t>
         </is>
@@ -1073,8 +1198,16 @@
           <t>අපි අද lunch ගන්න hotel එකට යමුද?</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>අපි අද lunch ගන්න hotel එකට යමුද?</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Isolated English Word Insertions in Singlish; Question forms</t>
@@ -1087,34 +1220,42 @@
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Neg_0018</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>mama heta morning shift eka innawa, eka nisaa ada night eke sleep karanna hithanawa.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>මම හෙට morning shift එක ඉන්නවා, ඒක නිසා අද night එකේ sleep කරන්න හිතනවා.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>මම හෙට morning shift එක ඉන්නවා, ඒක නිසා අද night එකේ sleep කරන්න හිතනවා.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Evidence: 'morning', 'shift', 'night', 'sleep' are isolated English words</t>
         </is>
@@ -1141,8 +1282,16 @@
           <t>මම අද ගොඩක් tired, so just chilling at home.</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>මම අද ගොඩක් tired, so just chilling at home.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Multi-Word English Phrases in Singlish</t>
@@ -1155,34 +1304,42 @@
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Neg_0020</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>api heta plan eka change karamu, let me know if that works for you.</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>අපි හෙට plan එක change කරමු, let me know if that works for you.</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>අපි හෙට plan එක change කරමු, let me know if that works for you.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Multi-Word English Phrases in Singlish; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'let me know if that works for you' is a full English phrase; 'plan', 'change' are isolated words</t>
         </is>
@@ -1209,8 +1366,16 @@
           <t>ඔයාගේ WiFi password එක මොකක්ද?</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>ඔයාගේ WiFi password එක මොකක්ද?</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>English Digital Terms in Singlish; Question forms</t>
@@ -1223,34 +1388,42 @@
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Neg_0022</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>mama software eka update karala restart dunna, ethakot system eka hang una.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>මම software එක update කරලා restart දුන්නා, එතකොට system එක hang උනා.</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>මම software එක update කරලා restart දුන්නා, එතකොට් system එක hang වුණා.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>English Digital Terms in Singlish</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Evidence: 'software', 'update', 'restart', 'system', 'hang' are digital terms</t>
         </is>
@@ -1277,8 +1450,16 @@
           <t>Facebook එකේ post එක share කරන්න.</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Facebook එකේ පෝස්ට් එක share කරන්න.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Platform/App Names in Singlish; Command forms</t>
@@ -1291,34 +1472,42 @@
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Neg_0024</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>oya Instagram story eka balawada? mama YouTube eke video ekak share karala thibba.</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>ඔයා Instagram story එක බලාවද? මම YouTube එකේ video එකක් share කරලා තිබ්බා.</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>ඔයා Instagram story එක බලවද? මම YouTube ඒකේ video එකක් share කරලා තිබ්බා.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Platform/App Names in Singlish; Question forms</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'Instagram', 'YouTube' are platform names; 'story', 'video', 'share' are digital terms</t>
         </is>
@@ -1345,8 +1534,16 @@
           <t>ASAP ඒක කරන්න, boss කිව්වා.</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>ASAP ඒක කරන්න, boss කිව්වා.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>English Abbreviations/Acronyms in Singlish; Isolated English Word Insertions in Singlish</t>
@@ -1359,34 +1556,42 @@
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Neg_0026</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>mama CV eka update karala HR kiyanawa, DNA report eka athi wenakam wait karanna.</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>මම CV එක update කරලා HR කියනවා, DNA report එක ඇති වෙනකම් wait කරන්න.</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>මම CV ඒක update කරලා HR කියනවා, DNA report එක ඇති වෙනකම් wait කරන්න.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>English Abbreviations/Acronyms in Singlish; English Digital Terms in Singlish</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'CV', 'HR', 'DNA' are abbreviations; 'update', 'report', 'wait' are English terms</t>
         </is>
@@ -1413,8 +1618,16 @@
           <t>හෙට uni එකේ exam එකක් තියෙනවා.</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>හෙට uni එකේ exam එකක් තියෙනවා.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>English Clipped Forms in Singlish</t>
@@ -1427,34 +1640,42 @@
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Neg_0028</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>gym eke bro eka kiwwa, promo eka ada vitharai kiyala, so api yamu.</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>gym එකේ bro එක කිව්වා, promo එක අද විතරයි කියලා, so අපි යමු.</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>gym එකේ bro එක කිව්වා, ප්රොමෝ එක අද විතරයි කියලා, සෝ අපි යමු.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>English Clipped Forms in Singlish; Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'gym' clipped, 'promo' clipped from 'promotion'; 'bro' is slang</t>
         </is>
@@ -1481,8 +1702,16 @@
           <t>අපි Kandy වලට යනවාද?</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>අපි Kandy වලට යනවද?</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Place Names Embedded in Singlish; Question forms</t>
@@ -1495,34 +1724,42 @@
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Neg_0030</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>mama Colombo eken Galle Face walata bus eken awa, methanin Galle Road eken yannam.</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>මම Colombo එකෙන් Galle Face වලට bus එකෙන් ආවා, මෙතනින් Galle Road එකෙන් යන්නම්.</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>මම Colombo එකෙන් Galle Face වලට bus එකෙන් ආවා, මෙතනින් Galle Road එකෙන් යන්නම්.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Place Names Embedded in Singlish; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'Colombo', 'Galle Face', 'Galle Road' are place names; 'bus' is English word</t>
         </is>
@@ -1549,8 +1786,16 @@
           <t>කමල් අයියා එන්න කිව්වද?</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>කමල් අයියා එන්න කිව්වද?</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Person Names Embedded in Singlish; Question forms</t>
@@ -1563,34 +1808,42 @@
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Neg_0032</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Nimal saha Sunil dennama late una, Priyanka witharai time eke awwe.</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>නිමල් සහ සුනිල් දෙන්නම late උනා, Priyanka විතරයි time එකේ ආව්වේ.</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>නිමල් සහ සුනිල් දෙන්නම late වුණා, ප්රියංකා විතරයි ටයිම් එකේ අව්වේ.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>UI Error</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>Person Names Embedded in Singlish; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'Nimal', 'Sunil', 'Priyanka' are person names; 'late', 'time' are English words</t>
         </is>
@@ -1617,8 +1870,16 @@
           <t>2nd floor එකේ room එක කොහෙද?</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>නිමල් සහ සුනිල් දෙන්නම late වුණා, ප්රියංකා විතරයි ටයිම් එකේ අව්වේ.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Inputs with Numbers and Numeric Suffixes; Question forms</t>
@@ -1631,34 +1892,42 @@
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Neg_0034</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>api 3rd dawasata plan karala tibba, ekath 4 denekma late una nisa cancel una.</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>අපි 3rd දවසට plan කරලා තිබ්බා, ඒකත් 4 දෙනෙක්ම late උනා නිසා cancel උනා.</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>2nd floor එකේ room එක කොහේද?</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Inputs with Numbers and Numeric Suffixes; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Rationale: '3rd' numeric suffix; 'plan', 'late', 'cancel' are English words</t>
         </is>
@@ -1685,8 +1954,16 @@
           <t>Rs. 500 දෙන්න පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 500 දෙන්න පුළුවන් ද?</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>UI Error</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Inputs with Currency; Question forms</t>
@@ -1699,34 +1976,42 @@
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Neg_0036</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>e jacket eka Rs. 3500 ta gatta, hari wadiya. USD 20 walata ganna puluwan una.</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>ඒ jacket එක Rs. 3500 ට ගත්තා, හරි වාඩියා. USD 20 වලට ගන්න පුළුවන් උනා.</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Rs. 500 දෙන්න පුළුවන් ද?</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>Inputs with Currency; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'Rs. 3500' and 'USD 20' are currency values; 'jacket' is English</t>
         </is>
@@ -1753,8 +2038,16 @@
           <t>meeting එක 9.30AM ට තිබ්බා.</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>meeting එක 9.30AM ට තිබ්බා.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>UI Error</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Inputs with Time Formats; Isolated English Word Insertions in Singlish</t>
@@ -1767,34 +2060,42 @@
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Neg_0038</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>bus eka 6:45PM ta enna one, mama 7:00PM walata station eke innakam wait karannm.</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>bus එක 6:45PM ට එන්න ඕනේ, මම 7:00PM වලට station එකේ ඉන්නකම් wait කරන්නම්.</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="3" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>meeting එක 9.30AM ට තිබ්බා.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>Inputs with Time Formats; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Rationale: '6:45PM' and '7:00PM' are time formats; 'bus', 'station', 'wait' are English</t>
         </is>
@@ -1821,8 +2122,16 @@
           <t>April 10 ට submit කරන්න ඕනේ.</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>අප්රේල් 10 ට submit කරන්න ඕනේ.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>UI Error</t>
+        </is>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Inputs with Dates; Command forms</t>
@@ -1835,34 +2144,42 @@
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Neg_0040</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>2026-03-15 ta confirm una, eka January 1 iden count karala 74 dawasak.</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>2026-03-15 ට confirm උනා, ඒක January 1 ඉදෙන් count කරලා 74 දවසක්.</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="3" t="inlineStr"/>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>අප්රේල් 10 ට submit කරන්න ඕනේ.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Inputs with Dates; Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Rationale: '2026-03-15' and 'January 1' are date formats; 'confirm', 'count' are English</t>
         </is>
@@ -1889,8 +2206,16 @@
           <t>ඒ gas cylinder එක kg 12ක් විතර.</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-15 ට confirm වුණා, ඒක ජනවාරි 1 ඉඩෙන් count කරලා 74 දවසක්.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Inputs with Unit of Measurements; Isolated English Word Insertions in Singlish</t>
@@ -1903,34 +2228,42 @@
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Neg_0042</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>mama km 5k withar dawasata walk karannawa, eka nisaa ada godak tired.</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>මම km 5ක් විතර දවසට walk කරනවා, ඒක නිසා අද ගොඩක් tired.</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>ඒ ගස් cylinder එක kg 12ක් විතර.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Inputs with Unit of Measurements; Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'km 5k' is unit of measurement; 'walk', 'tired' are English</t>
         </is>
@@ -1957,8 +2290,16 @@
           <t>අනේ bro, උඹ මාර යකෙක්ද!</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>මම km 5ක් විතර දවසට walk කරන්නවා, ඒක නිසා අද ගොඩක් තිරේද.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Inputs with Slang and Casual Phrasing; Isolated English Word Insertions in Singlish</t>
@@ -1971,34 +2312,42 @@
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Neg_0044</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>sirawata katta, uba api sette wela hadapu eka wadiya, elakiri machan!</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>සිරාවට කට්ටා, උඹ අපේ සෙට්ටේ වෙලා හැදෙපු එක වාඩියා, එළකිරි මචං!</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>අනේ bro, උඹ මාර යකෙක් ද!</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'sirawata', 'katta', 'elakiri', 'machan' are all slang/casual expressions</t>
         </is>
@@ -2025,8 +2374,16 @@
           <t>මේ link එක open කරන්න: www.google.lk</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>මේ link එක open කරන්න: www.google.lk</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Online Identifiers in Singlish; Command forms</t>
@@ -2039,34 +2396,42 @@
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Neg_0046</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>mata me email ekata file eka dannapan: test123@gmail.com, @Kasun ayya hodatama eka send karanna.</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>මට මේ email එකට file එක දන්නපං: test123@gmail.com, @Kasun අයියා හොඳටම ඒක send කරන්න.</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>මට මේ email එකට file එක දාන්නපන්: test123@gmail.com, @කසුන් අයියා හොදටම එක සෙන්ඩ් කරන්න.</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Online Identifiers in Singlish; Requests; Person Names Embedded in Singlish</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Rationale: 'test123@gmail.com' is email identifier; '@Kasun' is @mention; 'Kasun' is person name</t>
         </is>
@@ -2093,8 +2458,16 @@
           <t>මම ගොඩක් කැන්තිපි 😡 ඔයා එපා එපා කිව්වත්.</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>මම ගොඩක් කාන්තිපි 😡 ඔයා එපා එපා කිව්වෙත්.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Inputs Containing Emojis</t>
@@ -2107,34 +2480,42 @@
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Neg_0048</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>ada party eka mara hari una 🎉 hemoma awwa, Kamal aiyya witharai naththe 😢 ane.</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>අද party එක මාර හරි උනා 🎉 හෙමෝම ආව්වා, කමල් අයියා විතරයි නැත්තේ 😢 අනේ.</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="3" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>අද party එක මාර හරි උනා 🎉 හැමෝම අව්ව, කමල් අයියා විතරයි නැත්තේ 😢 අනේ.</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>Inputs Containing Emojis; Person Names Embedded in Singlish; Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Rationale: Contains 🎉 and 😢 emojis; 'Kamal' is person name; 'mara hari' is casual phrasing</t>
         </is>
@@ -2161,8 +2542,16 @@
           <t>මචං, අද අපි කියන ඒක වගේ තමයි උනේ. මම office එකෙන් 5:30PM ට පිට උනා, bus එක full නිසා Kandy road එකේ Rs. 200 taxi එකක් ගත්තා. නිමල් අයියා කිව්වා ASAP ගෙදර යන්න කියලා. මම 3rd time තමයි late වෙන්නේ. next time carpooling කරමු, ok ද bro?</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>මචං, අද අපි කියන එක වගේ තමයි උනේ. මම office එකෙන් 5:30PM ට පිට වුණා, bus එක full නිසා Kandy road එකේ Rs. 200 ටාක්සි එකක් ගත්තා. නිමල් අයියා කිව්වා ASAP ගෙදර යන්න කියලා. මම 3rd time තමයි late වෙන්නේ. next time carpooling කරමු, ඕක ද bro?</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>UI Error</t>
+        </is>
+      </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Inputs with Time Formats; Place Names Embedded in Singlish; Inputs with Currency; English Abbreviations/Acronyms in Singlish; Inputs with Numbers and Numeric Suffixes; Inputs with Slang and Casual Phrasing; Isolated English Word Insertions in Singlish; Person Names Embedded in Singlish</t>
@@ -2175,34 +2564,42 @@
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Neg_0050</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>ado bro 😅, mata ona une YouTube eke e tutorial eka, mama www.youtube.com baluwata eya delete karalaa. USD 10 dala premium gatta, ethakot 4K videos play wenne nae. mama IT support eka contact karala kiwwa 2026-04-01 iden fix wenawa kiyala. Kasun saha Dilshan dennama e same issue eke innawa. ASAP fix karanna puluwannama karanna, nathnam Rs. 1500 refund karanna one!</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>ආඩෝ bro 😅, මට ඕනේ උනේ YouTube එකේ ඒ tutorial එක, මම www.youtube.com බැලුවාට එයා delete කරලා. USD 10 දාලා premium ගත්තා, එතකොට 4K videos play වෙන්නේ නෑ. මම IT support එක contact කරලා කිව්වා 2026-04-01 ඉදෙන් fix වෙනවා කියලා. කාසුන් සහ දිල්ශාන් දෙන්නම ඒ same issue එකේ ඉන්නවා. ASAP fix කරන්න පුළුවන්නම් කරන්න, නැත්නම් Rs. 1500 refund කරන්න ඕනේ!</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>මචං, අද අපි කියන එක වගේ තමයි උනේ. මම office එකෙන් 5:30PM ට පිට වුණා, bus එක full නිසා Kandy road එකේ Rs. 200 ටාක්සි එකක් ගත්තා. නිමල් අයියා කිව්වා ASAP ගෙදර යන්න කියලා. මම 3rd time තමයි late වෙන්නේ. next time carpooling කරමු, ඕක ද bro?</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>Inputs Containing Emojis; Platform/App Names in Singlish; Online Identifiers in Singlish; Inputs with Currency; English Digital Terms in Singlish; Inputs with Dates; English Abbreviations/Acronyms in Singlish; Inputs with Slang and Casual Phrasing; Person Names Embedded in Singlish</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Rationale: Complex L-length covering 9 input types. '😅' emoji; 'YouTube' platform; 'www.youtube.com' URL; 'USD 10','Rs. 1500' currencies; 'premium','4K','videos' digital terms; '2026-04-01' date; 'ASAP' acronym; 'ado','bro' slang; 'Kasun','Dilshan' person names</t>
         </is>
@@ -2210,5 +2607,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>